<commit_message>
Direct Write Excel for BAND SAW-03 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_BAND SAW-03.xlsx
+++ b/FM-MN-07_BAND SAW-03.xlsx
@@ -1771,7 +1771,11 @@
       <c r="E6" s="29" t="inlineStr"/>
       <c r="F6" s="29" t="inlineStr"/>
       <c r="G6" s="29" t="inlineStr"/>
-      <c r="H6" s="29" t="inlineStr"/>
+      <c r="H6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="29" t="inlineStr"/>
       <c r="J6" s="29" t="inlineStr"/>
       <c r="K6" s="29" t="inlineStr"/>
@@ -1812,7 +1816,11 @@
       <c r="E7" s="29" t="inlineStr"/>
       <c r="F7" s="29" t="inlineStr"/>
       <c r="G7" s="29" t="inlineStr"/>
-      <c r="H7" s="29" t="inlineStr"/>
+      <c r="H7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="29" t="inlineStr"/>
       <c r="J7" s="29" t="inlineStr"/>
       <c r="K7" s="29" t="inlineStr"/>
@@ -1853,7 +1861,11 @@
       <c r="E8" s="29" t="inlineStr"/>
       <c r="F8" s="29" t="inlineStr"/>
       <c r="G8" s="29" t="inlineStr"/>
-      <c r="H8" s="29" t="inlineStr"/>
+      <c r="H8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="29" t="inlineStr"/>
       <c r="J8" s="29" t="inlineStr"/>
       <c r="K8" s="29" t="inlineStr"/>
@@ -1894,7 +1906,11 @@
       <c r="E9" s="29" t="inlineStr"/>
       <c r="F9" s="29" t="inlineStr"/>
       <c r="G9" s="29" t="inlineStr"/>
-      <c r="H9" s="29" t="inlineStr"/>
+      <c r="H9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="29" t="inlineStr"/>
       <c r="J9" s="29" t="inlineStr"/>
       <c r="K9" s="29" t="inlineStr"/>
@@ -1935,7 +1951,11 @@
       <c r="E10" s="29" t="inlineStr"/>
       <c r="F10" s="29" t="inlineStr"/>
       <c r="G10" s="29" t="inlineStr"/>
-      <c r="H10" s="29" t="inlineStr"/>
+      <c r="H10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="29" t="inlineStr"/>
       <c r="J10" s="29" t="inlineStr"/>
       <c r="K10" s="29" t="inlineStr"/>
@@ -1970,7 +1990,11 @@
       <c r="E11" s="40" t="inlineStr"/>
       <c r="F11" s="40" t="inlineStr"/>
       <c r="G11" s="40" t="inlineStr"/>
-      <c r="H11" s="40" t="inlineStr"/>
+      <c r="H11" s="41" t="inlineStr">
+        <is>
+          <t>วชิรทย์</t>
+        </is>
+      </c>
       <c r="I11" s="40" t="inlineStr"/>
       <c r="J11" s="40" t="inlineStr"/>
       <c r="K11" s="40" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for BAND SAW-03 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_BAND SAW-03.xlsx
+++ b/FM-MN-07_BAND SAW-03.xlsx
@@ -1776,7 +1776,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="29" t="inlineStr"/>
+      <c r="I6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="29" t="inlineStr"/>
       <c r="K6" s="29" t="inlineStr"/>
       <c r="L6" s="29" t="inlineStr"/>
@@ -1821,7 +1825,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="29" t="inlineStr"/>
+      <c r="I7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="29" t="inlineStr"/>
       <c r="K7" s="29" t="inlineStr"/>
       <c r="L7" s="29" t="inlineStr"/>
@@ -1866,7 +1874,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="29" t="inlineStr"/>
+      <c r="I8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="29" t="inlineStr"/>
       <c r="K8" s="29" t="inlineStr"/>
       <c r="L8" s="29" t="inlineStr"/>
@@ -1911,7 +1923,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="29" t="inlineStr"/>
+      <c r="I9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="29" t="inlineStr"/>
       <c r="K9" s="29" t="inlineStr"/>
       <c r="L9" s="29" t="inlineStr"/>
@@ -1956,7 +1972,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="29" t="inlineStr"/>
+      <c r="I10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="29" t="inlineStr"/>
       <c r="K10" s="29" t="inlineStr"/>
       <c r="L10" s="29" t="inlineStr"/>
@@ -1995,7 +2015,11 @@
           <t>วชิรทย์</t>
         </is>
       </c>
-      <c r="I11" s="40" t="inlineStr"/>
+      <c r="I11" s="41" t="inlineStr">
+        <is>
+          <t>วชิรทย์</t>
+        </is>
+      </c>
       <c r="J11" s="40" t="inlineStr"/>
       <c r="K11" s="40" t="inlineStr"/>
       <c r="L11" s="40" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for BAND SAW-03 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_BAND SAW-03.xlsx
+++ b/FM-MN-07_BAND SAW-03.xlsx
@@ -1781,7 +1781,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="29" t="inlineStr"/>
+      <c r="J6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="29" t="inlineStr"/>
       <c r="L6" s="29" t="inlineStr"/>
       <c r="M6" s="29" t="inlineStr"/>
@@ -1830,7 +1834,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="29" t="inlineStr"/>
+      <c r="J7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="29" t="inlineStr"/>
       <c r="L7" s="29" t="inlineStr"/>
       <c r="M7" s="29" t="inlineStr"/>
@@ -1879,7 +1887,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="29" t="inlineStr"/>
+      <c r="J8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="29" t="inlineStr"/>
       <c r="L8" s="29" t="inlineStr"/>
       <c r="M8" s="29" t="inlineStr"/>
@@ -1928,7 +1940,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="29" t="inlineStr"/>
+      <c r="J9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="29" t="inlineStr"/>
       <c r="L9" s="29" t="inlineStr"/>
       <c r="M9" s="29" t="inlineStr"/>
@@ -1977,7 +1993,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="29" t="inlineStr"/>
+      <c r="J10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="29" t="inlineStr"/>
       <c r="L10" s="29" t="inlineStr"/>
       <c r="M10" s="29" t="inlineStr"/>
@@ -2020,7 +2040,11 @@
           <t>วชิรทย์</t>
         </is>
       </c>
-      <c r="J11" s="40" t="inlineStr"/>
+      <c r="J11" s="41" t="inlineStr">
+        <is>
+          <t>วชิรวิทย์</t>
+        </is>
+      </c>
       <c r="K11" s="40" t="inlineStr"/>
       <c r="L11" s="40" t="inlineStr"/>
       <c r="M11" s="40" t="inlineStr"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for BAND SAW-03 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_BAND SAW-03.xlsx
+++ b/FM-MN-07_BAND SAW-03.xlsx
@@ -1787,7 +1787,11 @@
         </is>
       </c>
       <c r="K6" s="29" t="inlineStr"/>
-      <c r="L6" s="29" t="inlineStr"/>
+      <c r="L6" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="29" t="inlineStr"/>
       <c r="N6" s="29" t="inlineStr"/>
       <c r="O6" s="29" t="inlineStr"/>
@@ -1840,7 +1844,11 @@
         </is>
       </c>
       <c r="K7" s="29" t="inlineStr"/>
-      <c r="L7" s="29" t="inlineStr"/>
+      <c r="L7" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="29" t="inlineStr"/>
       <c r="N7" s="29" t="inlineStr"/>
       <c r="O7" s="29" t="inlineStr"/>
@@ -1893,7 +1901,11 @@
         </is>
       </c>
       <c r="K8" s="29" t="inlineStr"/>
-      <c r="L8" s="29" t="inlineStr"/>
+      <c r="L8" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="29" t="inlineStr"/>
       <c r="N8" s="29" t="inlineStr"/>
       <c r="O8" s="29" t="inlineStr"/>
@@ -1946,7 +1958,11 @@
         </is>
       </c>
       <c r="K9" s="29" t="inlineStr"/>
-      <c r="L9" s="29" t="inlineStr"/>
+      <c r="L9" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="29" t="inlineStr"/>
       <c r="N9" s="29" t="inlineStr"/>
       <c r="O9" s="29" t="inlineStr"/>
@@ -1999,7 +2015,11 @@
         </is>
       </c>
       <c r="K10" s="29" t="inlineStr"/>
-      <c r="L10" s="29" t="inlineStr"/>
+      <c r="L10" s="29" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="29" t="inlineStr"/>
       <c r="N10" s="29" t="inlineStr"/>
       <c r="O10" s="29" t="inlineStr"/>
@@ -2046,7 +2066,11 @@
         </is>
       </c>
       <c r="K11" s="40" t="inlineStr"/>
-      <c r="L11" s="40" t="inlineStr"/>
+      <c r="L11" s="41" t="inlineStr">
+        <is>
+          <t>วชิรวิย์</t>
+        </is>
+      </c>
       <c r="M11" s="40" t="inlineStr"/>
       <c r="N11" s="40" t="inlineStr"/>
       <c r="O11" s="40" t="inlineStr"/>

</xml_diff>